<commit_message>
Adding real customer to delete and trying to correct test name
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/testData.xlsx
+++ b/src/test/resources/excel/testData.xlsx
@@ -115,10 +115,10 @@
     <t>id</t>
   </si>
   <si>
-    <t>cus_USP7xrjMNFOwpa</t>
-  </si>
-  <si>
-    <t>cus_USP7u8ayA9AIky</t>
+    <t>cus_UVmI0qXnGkYsCn</t>
+  </si>
+  <si>
+    <t>cus_UVmIziufAYI5zE</t>
   </si>
 </sst>
 </file>

</xml_diff>